<commit_message>
Admin: edit data/events.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -929,9 +929,62 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v>Event</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Maharashtra Day</v>
+      </c>
+      <c r="D11" t="str">
+        <v>May</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>2026</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Split Shala Events into dedicated data/shala-events.xlsx; add Calendar to Shala sub-nav
- New data/shala-events.xlsx, fully independent from data/events.xlsx
- main.js renderShalaEvents() now reads SHALA_EVENTS_DB instead of
  filtering the shared Events sheet by Audience
- Removed the now-unused Audience column + validation from data/events.xlsx
- Registered data/shala-events.xlsx in admin-worker (XLSX_FILES + shala
  PAGES group), so the Shala role can manage it directly
- Updated README and in-code comments to match
- Added a Calendar link to the shala.html sub-nav
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="18" max="18"/>
@@ -537,11 +537,6 @@
           <t>Price Details</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Audience</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -1152,11 +1147,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"General,Shala"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>